<commit_message>
Dealer report page, fed from new withdrawals and dealers sheets
"ورود به گزارش" on the dealer picker now opens /dealer-report/<dealer>,
styled like the management dashboard: tank gauge, oil-remaining and
days-left rings, the injection control panel (display only, not connected
to the device), withdrawals for a chosen period, and monthly / weekly /
weekday / hourly / per-injection-size charts.

Data comes from two new workbook sheets, «نمایندگی‌ها» (tank capacity and
inventory) and «برداشت‌ها» (one row per withdrawal); the template has a
sample Partak log. Access is a new "dealers" page in the access table, and
data.php sends those users only these sheets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dst/lubestation-site/web/public/lubestation-data-template.xlsx
+++ b/dst/lubestation-site/web/public/lubestation-data-template.xlsx
@@ -12,7 +12,9 @@
     <sheet name="تجهیزات" sheetId="5" r:id="rId5"/>
     <sheet name="سرویس‌ها" sheetId="6" r:id="rId6"/>
     <sheet name="قطعات یدکی" sheetId="7" r:id="rId7"/>
-    <sheet name="تنظیمات" sheetId="8" r:id="rId8"/>
+    <sheet name="نمایندگی‌ها" sheetId="8" r:id="rId8"/>
+    <sheet name="برداشت‌ها" sheetId="9" r:id="rId9"/>
+    <sheet name="تنظیمات" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -132,8 +134,65 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t xml:space="preserve">برگهٔ «برداشت‌ها»: هر ردیف یک برداشت (تزریق) روغن در یک نمایندگی است. ساعت را به شکل 14:30 بنویسید. نام نمایندگی باید با برگهٔ «نمایندگی‌ها» یکی باشد.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">برگهٔ «نمایندگی‌ها»: ظرفیت و موجودی فعلی مخزن هر نمایندگی برای صفحهٔ «گزارش نمایندگی».</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t xml:space="preserve">این برگه (راهنما) توسط سایت خوانده نمی‌شود.</t>
         </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">عنوان</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">مقدار</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">زمان تأمین (روز)</t>
+        </is>
+      </c>
+      <c r="B2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">میانگین زمان رفع مشکل (روز)</t>
+        </is>
+      </c>
+      <c r="B3">
+        <v>3.2</v>
       </c>
     </row>
   </sheetData>
@@ -1430,40 +1489,3970 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">عنوان</t>
+          <t xml:space="preserve">نمایندگی</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t xml:space="preserve">مقدار</t>
+          <t xml:space="preserve">شهر</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ظرفیت مخزن (لیتر)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">موجودی فعلی (لیتر)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">زمان تأمین (روز)</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>21</v>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">اصفهان</t>
+        </is>
+      </c>
+      <c r="C2">
+        <v>6000</v>
+      </c>
+      <c r="D2">
+        <v>4210</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">میانگین زمان رفع مشکل (روز)</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>3.2</v>
+          <t xml:space="preserve">آریا دیزل تهران</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تهران</t>
+        </is>
+      </c>
+      <c r="C3">
+        <v>4000</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">کاویان روان تبریز</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تبریز</t>
+        </is>
+      </c>
+      <c r="C4">
+        <v>4000</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سپهر لوب شیراز</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">شیراز</t>
+        </is>
+      </c>
+      <c r="C5">
+        <v>4000</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1" style="2"/>
+    <col min="3" max="3" width="10" customWidth="1" style="2"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">نمایندگی</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">تاریخ</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">ساعت</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">مقدار (لیتر)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">دستگاه</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/12</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:57</t>
+        </is>
+      </c>
+      <c r="D2">
+        <v>11.2</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/12</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:21</t>
+        </is>
+      </c>
+      <c r="D3">
+        <v>40.6</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/12</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:24</t>
+        </is>
+      </c>
+      <c r="D4">
+        <v>34.3</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/14</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:14</t>
+        </is>
+      </c>
+      <c r="D5">
+        <v>16.9</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/14</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:23</t>
+        </is>
+      </c>
+      <c r="D6">
+        <v>17.5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/15</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:36</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>45.3</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/15</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:19</t>
+        </is>
+      </c>
+      <c r="D8">
+        <v>32.8</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/15</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:50</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>36</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/16</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:34</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>17.8</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/16</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:44</t>
+        </is>
+      </c>
+      <c r="D11">
+        <v>39.3</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:04</t>
+        </is>
+      </c>
+      <c r="D12">
+        <v>25.9</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:43</t>
+        </is>
+      </c>
+      <c r="D13">
+        <v>25.3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:00</t>
+        </is>
+      </c>
+      <c r="D14">
+        <v>48.3</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/18</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:21</t>
+        </is>
+      </c>
+      <c r="D15">
+        <v>38.8</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/18</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:01</t>
+        </is>
+      </c>
+      <c r="D16">
+        <v>47.5</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/18</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:06</t>
+        </is>
+      </c>
+      <c r="D17">
+        <v>38.7</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/18</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:43</t>
+        </is>
+      </c>
+      <c r="D18">
+        <v>25.5</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/19</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:26</t>
+        </is>
+      </c>
+      <c r="D19">
+        <v>39.9</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/19</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:40</t>
+        </is>
+      </c>
+      <c r="D20">
+        <v>19</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/19</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:42</t>
+        </is>
+      </c>
+      <c r="D21">
+        <v>48.8</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/19</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:08</t>
+        </is>
+      </c>
+      <c r="D22">
+        <v>42.2</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/19</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:28</t>
+        </is>
+      </c>
+      <c r="D23">
+        <v>16.7</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/21</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:45</t>
+        </is>
+      </c>
+      <c r="D24">
+        <v>42.8</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/22</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:24</t>
+        </is>
+      </c>
+      <c r="D25">
+        <v>25</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/22</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:57</t>
+        </is>
+      </c>
+      <c r="D26">
+        <v>34.1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/22</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:37</t>
+        </is>
+      </c>
+      <c r="D27">
+        <v>12.7</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/22</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:45</t>
+        </is>
+      </c>
+      <c r="D28">
+        <v>19.6</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/22</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:53</t>
+        </is>
+      </c>
+      <c r="D29">
+        <v>18.8</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/23</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:48</t>
+        </is>
+      </c>
+      <c r="D30">
+        <v>40.9</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/23</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:41</t>
+        </is>
+      </c>
+      <c r="D31">
+        <v>49.3</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/23</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:55</t>
+        </is>
+      </c>
+      <c r="D32">
+        <v>35.4</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/23</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:18</t>
+        </is>
+      </c>
+      <c r="D33">
+        <v>8.1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/24</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:53</t>
+        </is>
+      </c>
+      <c r="D34">
+        <v>21.2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/24</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:06</t>
+        </is>
+      </c>
+      <c r="D35">
+        <v>31.6</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/24</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:21</t>
+        </is>
+      </c>
+      <c r="D36">
+        <v>29.3</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/24</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:22</t>
+        </is>
+      </c>
+      <c r="D37">
+        <v>46</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/25</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:05</t>
+        </is>
+      </c>
+      <c r="D38">
+        <v>28.7</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/25</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:11</t>
+        </is>
+      </c>
+      <c r="D39">
+        <v>21.1</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/25</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:39</t>
+        </is>
+      </c>
+      <c r="D40">
+        <v>33.6</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/25</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:06</t>
+        </is>
+      </c>
+      <c r="D41">
+        <v>33.1</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/25</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:21</t>
+        </is>
+      </c>
+      <c r="D42">
+        <v>20.1</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/26</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:30</t>
+        </is>
+      </c>
+      <c r="D43">
+        <v>48.6</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/28</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:16</t>
+        </is>
+      </c>
+      <c r="D44">
+        <v>18.1</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/28</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:08</t>
+        </is>
+      </c>
+      <c r="D45">
+        <v>43.2</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/28</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:09</t>
+        </is>
+      </c>
+      <c r="D46">
+        <v>38.4</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/28</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:57</t>
+        </is>
+      </c>
+      <c r="D47">
+        <v>16.9</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/29</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:29</t>
+        </is>
+      </c>
+      <c r="D48">
+        <v>38</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/29</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:32</t>
+        </is>
+      </c>
+      <c r="D49">
+        <v>43.8</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/29</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:38</t>
+        </is>
+      </c>
+      <c r="D50">
+        <v>9.2</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/29</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:11</t>
+        </is>
+      </c>
+      <c r="D51">
+        <v>44.8</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/30</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:39</t>
+        </is>
+      </c>
+      <c r="D52">
+        <v>27.3</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/30</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:06</t>
+        </is>
+      </c>
+      <c r="D53">
+        <v>48.5</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/30</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="D54">
+        <v>46.9</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/31</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:31</t>
+        </is>
+      </c>
+      <c r="D55">
+        <v>10</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/31</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:35</t>
+        </is>
+      </c>
+      <c r="D56">
+        <v>27.1</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/31</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:53</t>
+        </is>
+      </c>
+      <c r="D57">
+        <v>19.8</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/31</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:58</t>
+        </is>
+      </c>
+      <c r="D58">
+        <v>12.4</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/06/31</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:33</t>
+        </is>
+      </c>
+      <c r="D59">
+        <v>17.6</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/01</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:35</t>
+        </is>
+      </c>
+      <c r="D60">
+        <v>24.7</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/02</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:32</t>
+        </is>
+      </c>
+      <c r="D61">
+        <v>40.1</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/02</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:36</t>
+        </is>
+      </c>
+      <c r="D62">
+        <v>36.9</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/02</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:21</t>
+        </is>
+      </c>
+      <c r="D63">
+        <v>48.5</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/04</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:08</t>
+        </is>
+      </c>
+      <c r="D64">
+        <v>46.3</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/04</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:57</t>
+        </is>
+      </c>
+      <c r="D65">
+        <v>23.5</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/04</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:57</t>
+        </is>
+      </c>
+      <c r="D66">
+        <v>17.7</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/04</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:15</t>
+        </is>
+      </c>
+      <c r="D67">
+        <v>32.7</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/04</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:25</t>
+        </is>
+      </c>
+      <c r="D68">
+        <v>21.9</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/05</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:02</t>
+        </is>
+      </c>
+      <c r="D69">
+        <v>44.6</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/05</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:07</t>
+        </is>
+      </c>
+      <c r="D70">
+        <v>50</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/05</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:16</t>
+        </is>
+      </c>
+      <c r="D71">
+        <v>22.3</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/05</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:42</t>
+        </is>
+      </c>
+      <c r="D72">
+        <v>11.4</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/05</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:24</t>
+        </is>
+      </c>
+      <c r="D73">
+        <v>37.8</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/06</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:28</t>
+        </is>
+      </c>
+      <c r="D74">
+        <v>33.8</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/06</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:38</t>
+        </is>
+      </c>
+      <c r="D75">
+        <v>47.2</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/07</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:03</t>
+        </is>
+      </c>
+      <c r="D76">
+        <v>15.3</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/07</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:50</t>
+        </is>
+      </c>
+      <c r="D77">
+        <v>19.3</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/07</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:35</t>
+        </is>
+      </c>
+      <c r="D78">
+        <v>27</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/08</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:13</t>
+        </is>
+      </c>
+      <c r="D79">
+        <v>11.6</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/08</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:34</t>
+        </is>
+      </c>
+      <c r="D80">
+        <v>37.8</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/09</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:27</t>
+        </is>
+      </c>
+      <c r="D81">
+        <v>22.3</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/09</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:29</t>
+        </is>
+      </c>
+      <c r="D82">
+        <v>12.7</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/09</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:22</t>
+        </is>
+      </c>
+      <c r="D83">
+        <v>47.2</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/09</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:05</t>
+        </is>
+      </c>
+      <c r="D84">
+        <v>46.2</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/11</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:05</t>
+        </is>
+      </c>
+      <c r="D85">
+        <v>21.6</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/11</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:33</t>
+        </is>
+      </c>
+      <c r="D86">
+        <v>42.9</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/11</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:48</t>
+        </is>
+      </c>
+      <c r="D87">
+        <v>37.6</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/11</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:22</t>
+        </is>
+      </c>
+      <c r="D88">
+        <v>22.4</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/11</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:45</t>
+        </is>
+      </c>
+      <c r="D89">
+        <v>27</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/12</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="D90">
+        <v>45.6</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/12</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:33</t>
+        </is>
+      </c>
+      <c r="D91">
+        <v>39.1</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/12</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:24</t>
+        </is>
+      </c>
+      <c r="D92">
+        <v>38.3</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/12</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:23</t>
+        </is>
+      </c>
+      <c r="D93">
+        <v>39.8</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/13</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:57</t>
+        </is>
+      </c>
+      <c r="D94">
+        <v>46.7</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/13</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:28</t>
+        </is>
+      </c>
+      <c r="D95">
+        <v>11</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/13</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:24</t>
+        </is>
+      </c>
+      <c r="D96">
+        <v>35.2</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/14</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:55</t>
+        </is>
+      </c>
+      <c r="D97">
+        <v>21.5</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/14</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:10</t>
+        </is>
+      </c>
+      <c r="D98">
+        <v>39.1</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/15</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:05</t>
+        </is>
+      </c>
+      <c r="D99">
+        <v>17.4</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/15</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:06</t>
+        </is>
+      </c>
+      <c r="D100">
+        <v>49.7</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/15</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:28</t>
+        </is>
+      </c>
+      <c r="D101">
+        <v>40.4</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/15</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:22</t>
+        </is>
+      </c>
+      <c r="D102">
+        <v>16.8</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/15</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:58</t>
+        </is>
+      </c>
+      <c r="D103">
+        <v>37.4</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/16</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:11</t>
+        </is>
+      </c>
+      <c r="D104">
+        <v>39.5</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/16</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:19</t>
+        </is>
+      </c>
+      <c r="D105">
+        <v>36</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/16</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:06</t>
+        </is>
+      </c>
+      <c r="D106">
+        <v>18.4</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/18</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:21</t>
+        </is>
+      </c>
+      <c r="D107">
+        <v>46.8</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/18</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:07</t>
+        </is>
+      </c>
+      <c r="D108">
+        <v>40.1</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/18</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:59</t>
+        </is>
+      </c>
+      <c r="D109">
+        <v>21.2</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/18</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:48</t>
+        </is>
+      </c>
+      <c r="D110">
+        <v>48.1</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/18</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:17</t>
+        </is>
+      </c>
+      <c r="D111">
+        <v>41.1</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/19</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:50</t>
+        </is>
+      </c>
+      <c r="D112">
+        <v>22.4</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/19</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:10</t>
+        </is>
+      </c>
+      <c r="D113">
+        <v>25.3</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/19</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:42</t>
+        </is>
+      </c>
+      <c r="D114">
+        <v>34.9</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/19</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:55</t>
+        </is>
+      </c>
+      <c r="D115">
+        <v>38.1</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/20</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:30</t>
+        </is>
+      </c>
+      <c r="D116">
+        <v>23.6</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/20</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:44</t>
+        </is>
+      </c>
+      <c r="D117">
+        <v>13.7</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/21</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="D118">
+        <v>15.5</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/21</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:53</t>
+        </is>
+      </c>
+      <c r="D119">
+        <v>18</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/21</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:22</t>
+        </is>
+      </c>
+      <c r="D120">
+        <v>45.6</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/21</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:18</t>
+        </is>
+      </c>
+      <c r="D121">
+        <v>40.2</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/21</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:59</t>
+        </is>
+      </c>
+      <c r="D122">
+        <v>31.9</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/22</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:19</t>
+        </is>
+      </c>
+      <c r="D123">
+        <v>21.2</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/22</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:52</t>
+        </is>
+      </c>
+      <c r="D124">
+        <v>29.2</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/22</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:44</t>
+        </is>
+      </c>
+      <c r="D125">
+        <v>35.4</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/22</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">17:46</t>
+        </is>
+      </c>
+      <c r="D126">
+        <v>13.4</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/23</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:20</t>
+        </is>
+      </c>
+      <c r="D127">
+        <v>27</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/23</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:22</t>
+        </is>
+      </c>
+      <c r="D128">
+        <v>21.3</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/23</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:00</t>
+        </is>
+      </c>
+      <c r="D129">
+        <v>39.3</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/23</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:02</t>
+        </is>
+      </c>
+      <c r="D130">
+        <v>37.8</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/23</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:15</t>
+        </is>
+      </c>
+      <c r="D131">
+        <v>30.7</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/25</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:03</t>
+        </is>
+      </c>
+      <c r="D132">
+        <v>34.5</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/25</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:27</t>
+        </is>
+      </c>
+      <c r="D133">
+        <v>22.3</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/25</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:46</t>
+        </is>
+      </c>
+      <c r="D134">
+        <v>9.6</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/26</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">10:12</t>
+        </is>
+      </c>
+      <c r="D135">
+        <v>19</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/26</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:34</t>
+        </is>
+      </c>
+      <c r="D136">
+        <v>14.7</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/27</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">08:25</t>
+        </is>
+      </c>
+      <c r="D137">
+        <v>15.8</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/27</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:51</t>
+        </is>
+      </c>
+      <c r="D138">
+        <v>37.9</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/27</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:25</t>
+        </is>
+      </c>
+      <c r="D139">
+        <v>14.2</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/28</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:32</t>
+        </is>
+      </c>
+      <c r="D140">
+        <v>38.8</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/28</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:35</t>
+        </is>
+      </c>
+      <c r="D141">
+        <v>16.2</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/29</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:44</t>
+        </is>
+      </c>
+      <c r="D142">
+        <v>44.3</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/29</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:08</t>
+        </is>
+      </c>
+      <c r="D143">
+        <v>24.3</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/07/30</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:58</t>
+        </is>
+      </c>
+      <c r="D144">
+        <v>47.5</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/02</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:07</t>
+        </is>
+      </c>
+      <c r="D145">
+        <v>24.6</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/02</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:17</t>
+        </is>
+      </c>
+      <c r="D146">
+        <v>46</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/03</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">07:39</t>
+        </is>
+      </c>
+      <c r="D147">
+        <v>41.1</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/04</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">16:13</t>
+        </is>
+      </c>
+      <c r="D148">
+        <v>42.8</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/05</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">11:10</t>
+        </is>
+      </c>
+      <c r="D149">
+        <v>21.6</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/05</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">12:27</t>
+        </is>
+      </c>
+      <c r="D150">
+        <v>27</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/05</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">13:42</t>
+        </is>
+      </c>
+      <c r="D151">
+        <v>34</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/05</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">14:09</t>
+        </is>
+      </c>
+      <c r="D152">
+        <v>23.3</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/06</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">09:14</t>
+        </is>
+      </c>
+      <c r="D153">
+        <v>25.2</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST2</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1405/08/06</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">15:30</t>
+        </is>
+      </c>
+      <c r="D154">
+        <v>22.3</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DST1</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
One dealer for Partak Sepehr / Partak Isfahan; no sample data locally
- The dealer is now named "پارتاک دیزل سپهر-اصفهان"; Excel rows under either
  old name merge into it (dealer aliases), so the dashboard no longer counts it twice
- Template regenerated with the new name
- The dev mock starts without the sample workbook, like a fresh host
  (LS_MOCK_SAMPLE=1 loads it), so local numbers match the real site

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dst/lubestation-site/web/public/lubestation-data-template.xlsx
+++ b/dst/lubestation-site/web/public/lubestation-data-template.xlsx
@@ -293,7 +293,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل سپهر</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -767,7 +767,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -799,7 +799,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -831,7 +831,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -863,7 +863,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1520,7 +1520,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1633,7 +1633,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="2">
@@ -1658,7 +1658,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="2">
@@ -1683,7 +1683,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="2">
@@ -1708,7 +1708,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="2">
@@ -1733,7 +1733,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B6" t="inlineStr" s="2">
@@ -1758,7 +1758,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B7" t="inlineStr" s="2">
@@ -1783,7 +1783,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="2">
@@ -1808,7 +1808,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="2">
@@ -1833,7 +1833,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B10" t="inlineStr" s="2">
@@ -1858,7 +1858,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="2">
@@ -1883,7 +1883,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="2">
@@ -1908,7 +1908,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="2">
@@ -1933,7 +1933,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="2">
@@ -1958,7 +1958,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="2">
@@ -1983,7 +1983,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="2">
@@ -2008,7 +2008,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B17" t="inlineStr" s="2">
@@ -2033,7 +2033,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B18" t="inlineStr" s="2">
@@ -2058,7 +2058,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B19" t="inlineStr" s="2">
@@ -2083,7 +2083,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B20" t="inlineStr" s="2">
@@ -2108,7 +2108,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B21" t="inlineStr" s="2">
@@ -2133,7 +2133,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B22" t="inlineStr" s="2">
@@ -2158,7 +2158,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B23" t="inlineStr" s="2">
@@ -2183,7 +2183,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B24" t="inlineStr" s="2">
@@ -2208,7 +2208,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B25" t="inlineStr" s="2">
@@ -2233,7 +2233,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B26" t="inlineStr" s="2">
@@ -2258,7 +2258,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B27" t="inlineStr" s="2">
@@ -2283,7 +2283,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B28" t="inlineStr" s="2">
@@ -2308,7 +2308,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B29" t="inlineStr" s="2">
@@ -2333,7 +2333,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B30" t="inlineStr" s="2">
@@ -2358,7 +2358,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B31" t="inlineStr" s="2">
@@ -2383,7 +2383,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B32" t="inlineStr" s="2">
@@ -2408,7 +2408,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B33" t="inlineStr" s="2">
@@ -2433,7 +2433,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B34" t="inlineStr" s="2">
@@ -2458,7 +2458,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B35" t="inlineStr" s="2">
@@ -2483,7 +2483,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B36" t="inlineStr" s="2">
@@ -2508,7 +2508,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B37" t="inlineStr" s="2">
@@ -2533,7 +2533,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B38" t="inlineStr" s="2">
@@ -2558,7 +2558,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B39" t="inlineStr" s="2">
@@ -2583,7 +2583,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B40" t="inlineStr" s="2">
@@ -2608,7 +2608,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B41" t="inlineStr" s="2">
@@ -2633,7 +2633,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B42" t="inlineStr" s="2">
@@ -2658,7 +2658,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B43" t="inlineStr" s="2">
@@ -2683,7 +2683,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B44" t="inlineStr" s="2">
@@ -2708,7 +2708,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B45" t="inlineStr" s="2">
@@ -2733,7 +2733,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B46" t="inlineStr" s="2">
@@ -2758,7 +2758,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B47" t="inlineStr" s="2">
@@ -2783,7 +2783,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B48" t="inlineStr" s="2">
@@ -2808,7 +2808,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B49" t="inlineStr" s="2">
@@ -2833,7 +2833,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B50" t="inlineStr" s="2">
@@ -2858,7 +2858,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B51" t="inlineStr" s="2">
@@ -2883,7 +2883,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B52" t="inlineStr" s="2">
@@ -2908,7 +2908,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B53" t="inlineStr" s="2">
@@ -2933,7 +2933,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B54" t="inlineStr" s="2">
@@ -2958,7 +2958,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B55" t="inlineStr" s="2">
@@ -2983,7 +2983,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B56" t="inlineStr" s="2">
@@ -3008,7 +3008,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B57" t="inlineStr" s="2">
@@ -3033,7 +3033,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B58" t="inlineStr" s="2">
@@ -3058,7 +3058,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B59" t="inlineStr" s="2">
@@ -3083,7 +3083,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B60" t="inlineStr" s="2">
@@ -3108,7 +3108,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B61" t="inlineStr" s="2">
@@ -3133,7 +3133,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B62" t="inlineStr" s="2">
@@ -3158,7 +3158,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B63" t="inlineStr" s="2">
@@ -3183,7 +3183,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B64" t="inlineStr" s="2">
@@ -3208,7 +3208,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B65" t="inlineStr" s="2">
@@ -3233,7 +3233,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B66" t="inlineStr" s="2">
@@ -3258,7 +3258,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B67" t="inlineStr" s="2">
@@ -3283,7 +3283,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B68" t="inlineStr" s="2">
@@ -3308,7 +3308,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B69" t="inlineStr" s="2">
@@ -3333,7 +3333,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B70" t="inlineStr" s="2">
@@ -3358,7 +3358,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B71" t="inlineStr" s="2">
@@ -3383,7 +3383,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B72" t="inlineStr" s="2">
@@ -3408,7 +3408,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B73" t="inlineStr" s="2">
@@ -3433,7 +3433,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B74" t="inlineStr" s="2">
@@ -3458,7 +3458,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B75" t="inlineStr" s="2">
@@ -3483,7 +3483,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B76" t="inlineStr" s="2">
@@ -3508,7 +3508,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B77" t="inlineStr" s="2">
@@ -3533,7 +3533,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B78" t="inlineStr" s="2">
@@ -3558,7 +3558,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B79" t="inlineStr" s="2">
@@ -3583,7 +3583,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B80" t="inlineStr" s="2">
@@ -3608,7 +3608,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B81" t="inlineStr" s="2">
@@ -3633,7 +3633,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B82" t="inlineStr" s="2">
@@ -3658,7 +3658,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B83" t="inlineStr" s="2">
@@ -3683,7 +3683,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B84" t="inlineStr" s="2">
@@ -3708,7 +3708,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B85" t="inlineStr" s="2">
@@ -3733,7 +3733,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B86" t="inlineStr" s="2">
@@ -3758,7 +3758,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B87" t="inlineStr" s="2">
@@ -3783,7 +3783,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B88" t="inlineStr" s="2">
@@ -3808,7 +3808,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B89" t="inlineStr" s="2">
@@ -3833,7 +3833,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B90" t="inlineStr" s="2">
@@ -3858,7 +3858,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B91" t="inlineStr" s="2">
@@ -3883,7 +3883,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B92" t="inlineStr" s="2">
@@ -3908,7 +3908,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B93" t="inlineStr" s="2">
@@ -3933,7 +3933,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B94" t="inlineStr" s="2">
@@ -3958,7 +3958,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B95" t="inlineStr" s="2">
@@ -3983,7 +3983,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B96" t="inlineStr" s="2">
@@ -4008,7 +4008,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B97" t="inlineStr" s="2">
@@ -4033,7 +4033,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B98" t="inlineStr" s="2">
@@ -4058,7 +4058,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B99" t="inlineStr" s="2">
@@ -4083,7 +4083,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B100" t="inlineStr" s="2">
@@ -4108,7 +4108,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B101" t="inlineStr" s="2">
@@ -4133,7 +4133,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B102" t="inlineStr" s="2">
@@ -4158,7 +4158,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B103" t="inlineStr" s="2">
@@ -4183,7 +4183,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B104" t="inlineStr" s="2">
@@ -4208,7 +4208,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B105" t="inlineStr" s="2">
@@ -4233,7 +4233,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B106" t="inlineStr" s="2">
@@ -4258,7 +4258,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B107" t="inlineStr" s="2">
@@ -4283,7 +4283,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B108" t="inlineStr" s="2">
@@ -4308,7 +4308,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B109" t="inlineStr" s="2">
@@ -4333,7 +4333,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B110" t="inlineStr" s="2">
@@ -4358,7 +4358,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B111" t="inlineStr" s="2">
@@ -4383,7 +4383,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B112" t="inlineStr" s="2">
@@ -4408,7 +4408,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B113" t="inlineStr" s="2">
@@ -4433,7 +4433,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B114" t="inlineStr" s="2">
@@ -4458,7 +4458,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B115" t="inlineStr" s="2">
@@ -4483,7 +4483,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B116" t="inlineStr" s="2">
@@ -4508,7 +4508,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B117" t="inlineStr" s="2">
@@ -4533,7 +4533,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B118" t="inlineStr" s="2">
@@ -4558,7 +4558,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B119" t="inlineStr" s="2">
@@ -4583,7 +4583,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B120" t="inlineStr" s="2">
@@ -4608,7 +4608,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B121" t="inlineStr" s="2">
@@ -4633,7 +4633,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B122" t="inlineStr" s="2">
@@ -4658,7 +4658,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B123" t="inlineStr" s="2">
@@ -4683,7 +4683,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B124" t="inlineStr" s="2">
@@ -4708,7 +4708,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B125" t="inlineStr" s="2">
@@ -4733,7 +4733,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B126" t="inlineStr" s="2">
@@ -4758,7 +4758,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B127" t="inlineStr" s="2">
@@ -4783,7 +4783,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B128" t="inlineStr" s="2">
@@ -4808,7 +4808,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B129" t="inlineStr" s="2">
@@ -4833,7 +4833,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B130" t="inlineStr" s="2">
@@ -4858,7 +4858,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B131" t="inlineStr" s="2">
@@ -4883,7 +4883,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B132" t="inlineStr" s="2">
@@ -4908,7 +4908,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B133" t="inlineStr" s="2">
@@ -4933,7 +4933,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B134" t="inlineStr" s="2">
@@ -4958,7 +4958,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B135" t="inlineStr" s="2">
@@ -4983,7 +4983,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B136" t="inlineStr" s="2">
@@ -5008,7 +5008,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B137" t="inlineStr" s="2">
@@ -5033,7 +5033,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B138" t="inlineStr" s="2">
@@ -5058,7 +5058,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B139" t="inlineStr" s="2">
@@ -5083,7 +5083,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B140" t="inlineStr" s="2">
@@ -5108,7 +5108,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B141" t="inlineStr" s="2">
@@ -5133,7 +5133,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B142" t="inlineStr" s="2">
@@ -5158,7 +5158,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B143" t="inlineStr" s="2">
@@ -5183,7 +5183,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B144" t="inlineStr" s="2">
@@ -5208,7 +5208,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B145" t="inlineStr" s="2">
@@ -5233,7 +5233,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B146" t="inlineStr" s="2">
@@ -5258,7 +5258,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B147" t="inlineStr" s="2">
@@ -5283,7 +5283,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B148" t="inlineStr" s="2">
@@ -5308,7 +5308,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B149" t="inlineStr" s="2">
@@ -5333,7 +5333,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B150" t="inlineStr" s="2">
@@ -5358,7 +5358,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B151" t="inlineStr" s="2">
@@ -5383,7 +5383,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B152" t="inlineStr" s="2">
@@ -5408,7 +5408,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B153" t="inlineStr" s="2">
@@ -5433,7 +5433,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t xml:space="preserve">پارتاک دیزل اصفهان</t>
+          <t xml:space="preserve">پارتاک دیزل سپهر-اصفهان</t>
         </is>
       </c>
       <c r="B154" t="inlineStr" s="2">

</xml_diff>